<commit_message>
Dodanie historii i raportów dotyczących importów
</commit_message>
<xml_diff>
--- a/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
+++ b/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\drukibaza\krakow\biblioteka\importer\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF397B6D-E8C1-4B61-9065-E70DD1637106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF179CA7-1496-4EEF-A073-33D9A6D47CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Rekordy" sheetId="1" r:id="rId1"/>
     <sheet name="Egzemplarze" sheetId="2" r:id="rId2"/>
     <sheet name="Załączniki" sheetId="4" r:id="rId3"/>
-    <sheet name="_Słowniki" sheetId="5" r:id="rId4"/>
+    <sheet name="_Słowniki" sheetId="5" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="CZCIONKI">_Słowniki!$C$2:$C$500</definedName>
@@ -2678,7 +2678,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="7">
     <dataValidation type="list" sqref="H2412:H5003" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"łaciński,polski,niemiecki,włoski,francuski,grecki,hebrajski,czeski,węgierski,inny"</formula1>
     </dataValidation>
@@ -2688,7 +2688,7 @@
     <dataValidation type="list" sqref="AF14:AF5003" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"opracowany,częściowo opracowany,nieopracowany"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="I15:I1482" xr:uid="{74CFD07B-3C15-4FD6-80BB-63D353764E3F}">
+    <dataValidation type="list" sqref="I14:I1482" xr:uid="{74CFD07B-3C15-4FD6-80BB-63D353764E3F}">
       <formula1>FORMATY</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="B10:B11" xr:uid="{FD3CE61B-BCC2-4A82-8782-18C5C0713060}">
@@ -2696,9 +2696,6 @@
     </dataValidation>
     <dataValidation type="list" sqref="H14:H2411" xr:uid="{B30642A1-54E9-46E7-8683-861F484FCE2B}">
       <formula1>JEZYKI</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="I14" xr:uid="{3368A8DE-0CFE-4EB3-B058-37A91C8B5651}">
-      <formula1>FORMATY</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M14:M2415" xr:uid="{670B3ECF-C9E3-469B-BC9D-75FBC2A7A4F0}">
       <formula1>CZCIONKI</formula1>

</xml_diff>

<commit_message>
Dodanie pierwszego poziomu walidacji do raportu (errors)
</commit_message>
<xml_diff>
--- a/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
+++ b/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\drukibaza\krakow\biblioteka\importer\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF179CA7-1496-4EEF-A073-33D9A6D47CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFA187C-DE38-421B-A606-7AA68AC903E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="102">
   <si>
     <t>Przed rozpoczęciem pracy pobierz najnowszy szablon BIF z BiDO (docelowo stały permalink).</t>
   </si>
@@ -179,300 +179,6 @@
   </si>
   <si>
     <t>częściowo opracowany</t>
-  </si>
-  <si>
-    <t>R000002</t>
-  </si>
-  <si>
-    <t>R000003</t>
-  </si>
-  <si>
-    <t>R000005</t>
-  </si>
-  <si>
-    <t>R000006</t>
-  </si>
-  <si>
-    <t>R000007</t>
-  </si>
-  <si>
-    <t>R000008</t>
-  </si>
-  <si>
-    <t>R000009</t>
-  </si>
-  <si>
-    <t>R000010</t>
-  </si>
-  <si>
-    <t>R000011</t>
-  </si>
-  <si>
-    <t>R000012</t>
-  </si>
-  <si>
-    <t>R000013</t>
-  </si>
-  <si>
-    <t>R000014</t>
-  </si>
-  <si>
-    <t>R000015</t>
-  </si>
-  <si>
-    <t>R000016</t>
-  </si>
-  <si>
-    <t>R000017</t>
-  </si>
-  <si>
-    <t>R000018</t>
-  </si>
-  <si>
-    <t>R000019</t>
-  </si>
-  <si>
-    <t>R000020</t>
-  </si>
-  <si>
-    <t>R000021</t>
-  </si>
-  <si>
-    <t>R000022</t>
-  </si>
-  <si>
-    <t>R000023</t>
-  </si>
-  <si>
-    <t>R000024</t>
-  </si>
-  <si>
-    <t>R000025</t>
-  </si>
-  <si>
-    <t>R000026</t>
-  </si>
-  <si>
-    <t>R000027</t>
-  </si>
-  <si>
-    <t>R000028</t>
-  </si>
-  <si>
-    <t>R000029</t>
-  </si>
-  <si>
-    <t>R000030</t>
-  </si>
-  <si>
-    <t>R000031</t>
-  </si>
-  <si>
-    <t>R000032</t>
-  </si>
-  <si>
-    <t>R000033</t>
-  </si>
-  <si>
-    <t>R000034</t>
-  </si>
-  <si>
-    <t>R000035</t>
-  </si>
-  <si>
-    <t>R000036</t>
-  </si>
-  <si>
-    <t>R000037</t>
-  </si>
-  <si>
-    <t>R000038</t>
-  </si>
-  <si>
-    <t>R000039</t>
-  </si>
-  <si>
-    <t>R000040</t>
-  </si>
-  <si>
-    <t>R000041</t>
-  </si>
-  <si>
-    <t>R000042</t>
-  </si>
-  <si>
-    <t>R000043</t>
-  </si>
-  <si>
-    <t>R000044</t>
-  </si>
-  <si>
-    <t>R000045</t>
-  </si>
-  <si>
-    <t>R000046</t>
-  </si>
-  <si>
-    <t>R000047</t>
-  </si>
-  <si>
-    <t>R000048</t>
-  </si>
-  <si>
-    <t>R000049</t>
-  </si>
-  <si>
-    <t>R000050</t>
-  </si>
-  <si>
-    <t>R000051</t>
-  </si>
-  <si>
-    <t>R000052</t>
-  </si>
-  <si>
-    <t>R000053</t>
-  </si>
-  <si>
-    <t>R000054</t>
-  </si>
-  <si>
-    <t>R000055</t>
-  </si>
-  <si>
-    <t>R000056</t>
-  </si>
-  <si>
-    <t>R000057</t>
-  </si>
-  <si>
-    <t>R000058</t>
-  </si>
-  <si>
-    <t>R000059</t>
-  </si>
-  <si>
-    <t>R000060</t>
-  </si>
-  <si>
-    <t>R000061</t>
-  </si>
-  <si>
-    <t>R000062</t>
-  </si>
-  <si>
-    <t>R000063</t>
-  </si>
-  <si>
-    <t>R000064</t>
-  </si>
-  <si>
-    <t>R000065</t>
-  </si>
-  <si>
-    <t>R000066</t>
-  </si>
-  <si>
-    <t>R000067</t>
-  </si>
-  <si>
-    <t>R000068</t>
-  </si>
-  <si>
-    <t>R000069</t>
-  </si>
-  <si>
-    <t>R000070</t>
-  </si>
-  <si>
-    <t>R000071</t>
-  </si>
-  <si>
-    <t>R000072</t>
-  </si>
-  <si>
-    <t>R000073</t>
-  </si>
-  <si>
-    <t>R000074</t>
-  </si>
-  <si>
-    <t>R000075</t>
-  </si>
-  <si>
-    <t>R000076</t>
-  </si>
-  <si>
-    <t>R000077</t>
-  </si>
-  <si>
-    <t>R000078</t>
-  </si>
-  <si>
-    <t>R000079</t>
-  </si>
-  <si>
-    <t>R000080</t>
-  </si>
-  <si>
-    <t>R000081</t>
-  </si>
-  <si>
-    <t>R000082</t>
-  </si>
-  <si>
-    <t>R000083</t>
-  </si>
-  <si>
-    <t>R000084</t>
-  </si>
-  <si>
-    <t>R000085</t>
-  </si>
-  <si>
-    <t>R000086</t>
-  </si>
-  <si>
-    <t>R000087</t>
-  </si>
-  <si>
-    <t>R000088</t>
-  </si>
-  <si>
-    <t>R000089</t>
-  </si>
-  <si>
-    <t>R000090</t>
-  </si>
-  <si>
-    <t>R000091</t>
-  </si>
-  <si>
-    <t>R000092</t>
-  </si>
-  <si>
-    <t>R000093</t>
-  </si>
-  <si>
-    <t>R000094</t>
-  </si>
-  <si>
-    <t>R000095</t>
-  </si>
-  <si>
-    <t>R000096</t>
-  </si>
-  <si>
-    <t>R000097</t>
-  </si>
-  <si>
-    <t>R000098</t>
-  </si>
-  <si>
-    <t>R000099</t>
-  </si>
-  <si>
-    <t>R000100</t>
   </si>
   <si>
     <t>Każdy egzemplarz = osobny wiersz. Powtarzaj ten sam ID importu, gdy wprowadzasz kilkaegzemplarzy dla tej samej edycji.</t>
@@ -1720,7 +1426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH115"/>
+  <dimension ref="A1:AH16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" customWidth="1"/>
@@ -1760,7 +1466,7 @@
   <sheetData>
     <row r="1" spans="1:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>174</v>
+        <v>76</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="32"/>
@@ -1794,7 +1500,7 @@
     </row>
     <row r="3" spans="1:34" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>172</v>
+        <v>74</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
@@ -1818,7 +1524,7 @@
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>167</v>
+        <v>69</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="3"/>
@@ -1835,7 +1541,7 @@
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
-        <v>168</v>
+        <v>70</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="3"/>
@@ -1886,7 +1592,7 @@
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" s="40" t="s">
-        <v>184</v>
+        <v>86</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="3"/>
@@ -1903,7 +1609,7 @@
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>176</v>
+        <v>78</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="3"/>
@@ -1920,7 +1626,7 @@
     </row>
     <row r="10" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>185</v>
+        <v>87</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="22"/>
@@ -1941,7 +1647,7 @@
     </row>
     <row r="11" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
-        <v>173</v>
+        <v>75</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="22"/>
@@ -1962,7 +1668,7 @@
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>169</v>
+        <v>71</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="3"/>
@@ -2063,7 +1769,7 @@
         <v>30</v>
       </c>
       <c r="AC14" s="38" t="s">
-        <v>180</v>
+        <v>82</v>
       </c>
       <c r="AD14" s="38" t="s">
         <v>31</v>
@@ -2078,7 +1784,7 @@
         <v>34</v>
       </c>
       <c r="AH14" s="8" t="s">
-        <v>175</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:34" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -2086,13 +1792,13 @@
         <v>35</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>188</v>
+        <v>90</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>186</v>
+        <v>88</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>187</v>
+        <v>89</v>
       </c>
       <c r="E15" s="6">
         <v>1586</v>
@@ -2101,10 +1807,10 @@
         <v>36</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>189</v>
+        <v>91</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>170</v>
+        <v>72</v>
       </c>
       <c r="I15" s="6">
         <v>4</v>
@@ -2113,41 +1819,41 @@
         <v>2</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>190</v>
+        <v>92</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
       <c r="M15" s="6" t="s">
         <v>37</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
       <c r="O15" s="7"/>
       <c r="P15" s="6" t="s">
-        <v>199</v>
+        <v>101</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>193</v>
+        <v>95</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>194</v>
+        <v>96</v>
       </c>
       <c r="S15" s="6" t="s">
         <v>38</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>195</v>
+        <v>97</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>198</v>
+        <v>100</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>196</v>
+        <v>98</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>197</v>
+        <v>99</v>
       </c>
       <c r="Y15" s="6" t="s">
         <v>39</v>
@@ -2165,7 +1871,7 @@
         <v>43</v>
       </c>
       <c r="AD15" s="39" t="s">
-        <v>181</v>
+        <v>83</v>
       </c>
       <c r="AE15" s="6" t="s">
         <v>44</v>
@@ -2174,507 +1880,12 @@
         <v>45</v>
       </c>
       <c r="AH15" s="6" t="s">
-        <v>159</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -2722,7 +1933,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>174</v>
+        <v>76</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="32"/>
@@ -2733,7 +1944,7 @@
     </row>
     <row r="2" spans="1:32" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>144</v>
+        <v>46</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="4"/>
@@ -2744,7 +1955,7 @@
     </row>
     <row r="3" spans="1:32" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>172</v>
+        <v>74</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="18"/>
@@ -2761,7 +1972,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>145</v>
+        <v>47</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="3"/>
@@ -2775,22 +1986,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>146</v>
+        <v>48</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>147</v>
+        <v>49</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>148</v>
+        <v>50</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>149</v>
+        <v>51</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>150</v>
+        <v>52</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>151</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
@@ -2798,22 +2009,22 @@
         <v>35</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>152</v>
+        <v>54</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>153</v>
+        <v>55</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>154</v>
+        <v>56</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>155</v>
+        <v>57</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>156</v>
+        <v>58</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>157</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2838,7 +2049,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>174</v>
+        <v>76</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="30"/>
@@ -2849,7 +2060,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>160</v>
+        <v>62</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="4"/>
@@ -2860,7 +2071,7 @@
     </row>
     <row r="3" spans="1:32" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>172</v>
+        <v>74</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
@@ -2877,7 +2088,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>171</v>
+        <v>73</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="4"/>
@@ -2888,7 +2099,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>178</v>
+        <v>80</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="4"/>
@@ -2899,7 +2110,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>179</v>
+        <v>81</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="4"/>
@@ -2913,22 +2124,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>161</v>
+        <v>63</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>162</v>
+        <v>64</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>163</v>
+        <v>65</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>158</v>
+        <v>60</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>164</v>
+        <v>66</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>177</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
@@ -2936,16 +2147,16 @@
         <v>35</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>165</v>
+        <v>67</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>151</v>
+        <v>53</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>163</v>
+        <v>65</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>166</v>
+        <v>68</v>
       </c>
       <c r="F15" s="7">
         <v>1</v>
@@ -2968,10 +2179,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>183</v>
+        <v>85</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Dodanie nowej funkcji walidacji błędów krytycznych 1
</commit_message>
<xml_diff>
--- a/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
+++ b/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\drukibaza\krakow\biblioteka\importer\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFA187C-DE38-421B-A606-7AA68AC903E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A548A1-24D4-48C7-99B8-771BDCA92370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rekordy" sheetId="1" r:id="rId1"/>
@@ -2163,10 +2163,11 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="B3:B5008 C3:C5006" xr:uid="{00000000-0002-0000-0300-000000000000}">
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="B3:B5008 C3:C13 C3631:C5006" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"ozdobniki,ryciny,uwagi,literatura_przedmiotu,marginalia"</formula1>
     </dataValidation>
+    <dataValidation sqref="C14:C3630" xr:uid="{BB998CE7-A26A-46FB-8975-C0A70F3DB3F4}"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Usprawniono i uzupełniono funkcje fuzzy i mechanizm ostrzeżeń w imporcie
</commit_message>
<xml_diff>
--- a/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
+++ b/biblioteka/importer/resources/formularz importu_BiDO_pusty.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\drukibaza\krakow\biblioteka\importer\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A548A1-24D4-48C7-99B8-771BDCA92370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11C28DC-E891-47BF-AC48-79C9886AE77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rekordy" sheetId="1" r:id="rId1"/>
@@ -184,9 +184,6 @@
     <t>Każdy egzemplarz = osobny wiersz. Powtarzaj ten sam ID importu, gdy wprowadzasz kilkaegzemplarzy dla tej samej edycji.</t>
   </si>
   <si>
-    <t>Jeżeli element istnieje, lecz nie został opisany, wpisz np. "Posiada marginalia – do uzupełnienia" (w przypadku marginaliów model odczyta nieuzupełnnione pole jako "brak właściwości").</t>
-  </si>
-  <si>
     <t>Biblioteka</t>
   </si>
   <si>
@@ -831,6 +828,9 @@
   </si>
   <si>
     <t>czcionka: a 111/20</t>
+  </si>
+  <si>
+    <t>Jeżeli element istnieje, lecz nie został opisany, wpisz np. "Posiada marginalia – do uzupełnienia" (w przypadku marginaliów model odczyta nieuzupełnione pole jako "brak właściwości").</t>
   </si>
 </sst>
 </file>
@@ -1466,7 +1466,7 @@
   <sheetData>
     <row r="1" spans="1:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="32"/>
@@ -1500,7 +1500,7 @@
     </row>
     <row r="3" spans="1:34" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
@@ -1524,7 +1524,7 @@
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="3"/>
@@ -1541,7 +1541,7 @@
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="3"/>
@@ -1592,7 +1592,7 @@
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" s="40" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="3"/>
@@ -1609,7 +1609,7 @@
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="3"/>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="10" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="22"/>
@@ -1647,7 +1647,7 @@
     </row>
     <row r="11" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="22"/>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="3"/>
@@ -1769,7 +1769,7 @@
         <v>30</v>
       </c>
       <c r="AC14" s="38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD14" s="38" t="s">
         <v>31</v>
@@ -1784,7 +1784,7 @@
         <v>34</v>
       </c>
       <c r="AH14" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:34" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1792,13 +1792,13 @@
         <v>35</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="E15" s="6">
         <v>1586</v>
@@ -1807,10 +1807,10 @@
         <v>36</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I15" s="6">
         <v>4</v>
@@ -1819,41 +1819,41 @@
         <v>2</v>
       </c>
       <c r="K15" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="L15" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="M15" s="6" t="s">
         <v>37</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O15" s="7"/>
       <c r="P15" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q15" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="R15" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="R15" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="S15" s="6" t="s">
         <v>38</v>
       </c>
       <c r="T15" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="U15" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="V15" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="U15" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="V15" s="6" t="s">
+      <c r="W15" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="W15" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="Y15" s="6" t="s">
         <v>39</v>
@@ -1871,7 +1871,7 @@
         <v>43</v>
       </c>
       <c r="AD15" s="39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AE15" s="6" t="s">
         <v>44</v>
@@ -1880,7 +1880,7 @@
         <v>45</v>
       </c>
       <c r="AH15" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -1933,7 +1933,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="32"/>
@@ -1955,7 +1955,7 @@
     </row>
     <row r="3" spans="1:32" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="18"/>
@@ -1972,7 +1972,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>101</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="3"/>
@@ -1986,22 +1986,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="G14" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
@@ -2009,22 +2009,22 @@
         <v>35</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="G15" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2049,7 +2049,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="30"/>
@@ -2060,7 +2060,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="4"/>
@@ -2071,7 +2071,7 @@
     </row>
     <row r="3" spans="1:32" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
@@ -2088,7 +2088,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="4"/>
@@ -2099,7 +2099,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="4"/>
@@ -2110,7 +2110,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="4"/>
@@ -2124,22 +2124,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>66</v>
-      </c>
       <c r="G14" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
@@ -2147,16 +2147,16 @@
         <v>35</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="F15" s="7">
         <v>1</v>
@@ -2180,10 +2180,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>15</v>

</xml_diff>